<commit_message>
Release JobRadar desktop career command center
</commit_message>
<xml_diff>
--- a/Python/JobRadar/reports/skill_gap_analysis.xlsx
+++ b/Python/JobRadar/reports/skill_gap_analysis.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -463,11 +463,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,40 +479,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cpq</t>
+          <t>Data Cloud</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Review or build a small proof-of-skill project for Cpq</t>
+          <t>Review or build a small proof-of-skill project for Data Cloud</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Data Cloud</t>
+          <t>Cpq</t>
         </is>
       </c>
       <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Review or build a small proof-of-skill project for Cpq</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Agentforce</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Review or build a small proof-of-skill project for Data Cloud</t>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Review or build a small proof-of-skill project for Agentforce</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Release JobRadar v2.7 apply-ready workflow
</commit_message>
<xml_diff>
--- a/Python/JobRadar/reports/skill_gap_analysis.xlsx
+++ b/Python/JobRadar/reports/skill_gap_analysis.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -459,51 +459,51 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Revenue Operations</t>
+          <t>Data Cloud</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Review or build a small proof-of-skill project for Revenue Operations</t>
+          <t>Review or build a small proof-of-skill project for Data Cloud</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Data Cloud</t>
+          <t>Revenue Operations</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Review or build a small proof-of-skill project for Data Cloud</t>
+          <t>Review or build a small proof-of-skill project for Revenue Operations</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cpq</t>
+          <t>Service Cloud</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Review or build a small proof-of-skill project for Cpq</t>
+          <t>Review or build a small proof-of-skill project for Service Cloud</t>
         </is>
       </c>
     </row>
@@ -533,6 +533,26 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>Review or build a small proof-of-skill project for Agentforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cpq</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Review or build a small proof-of-skill project for Cpq</t>
         </is>
       </c>
     </row>

</xml_diff>